<commit_message>
saving table2 yields as csv
</commit_message>
<xml_diff>
--- a/Output/EMMA-uncertainty/EMMA-mixing-fractions-uncertainty.xlsx
+++ b/Output/EMMA-uncertainty/EMMA-mixing-fractions-uncertainty.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="S Table 2. Hungerfod Feb ROS" sheetId="1" state="visible" r:id="rId3"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="141">
   <si>
     <t xml:space="preserve">Sample ID</t>
   </si>
@@ -87,6 +87,81 @@
     <t xml:space="preserve">2023-02-11 12:30:00</t>
   </si>
   <si>
+    <t xml:space="preserve">Groundwater</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Snowmelt lysimeter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soil water lysimeter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Groundwater_Uncertainty_95sig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Snowmelt lysimeter_Uncertainty_95sig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soil water lysimeter_Uncertainty_95sig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.640563e-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.545576e-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.742405e+00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.507713e-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.182702e-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.067480e-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.498535e+01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.442710e+01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.885781e-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.164136e-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.827733e+01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.785753e+01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.928295e-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.232444e-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.672211e-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.399861e-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NaN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.036609e-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.649435e+00</t>
+  </si>
+  <si>
     <t xml:space="preserve">RI23-1035</t>
   </si>
   <si>
@@ -147,15 +222,9 @@
     <t xml:space="preserve">2023-03-24 15:45:00</t>
   </si>
   <si>
-    <t xml:space="preserve">Groundwater_Uncertainty_95sig</t>
-  </si>
-  <si>
     <t xml:space="preserve">Meltwater_Uncertainty_95sig</t>
   </si>
   <si>
-    <t xml:space="preserve">Soil water lysimeter_Uncertainty_95sig</t>
-  </si>
-  <si>
     <t xml:space="preserve">RI23-1085</t>
   </si>
   <si>
@@ -274,15 +343,6 @@
   </si>
   <si>
     <t xml:space="preserve">RI23-1059</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Groundwater</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Snowmelt lysimeter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Soil water lysimeter</t>
   </si>
   <si>
     <t xml:space="preserve">RI23-1064</t>
@@ -662,7 +722,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.6"/>
@@ -860,67 +920,249 @@
       <c r="E8" s="2"/>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
+    <row r="9" customFormat="false" ht="46.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="2"/>
+      <c r="A10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>0.145442</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>2.742405</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="2"/>
+      <c r="A11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>0.393252</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>1.694802</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="2"/>
+      <c r="A12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>1.937141</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="2"/>
+      <c r="A13" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>0.957676</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0.000507</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
+      <c r="A14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>3.649435</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D16" s="0" t="n">
+        <f aca="false">D10/G10</f>
+        <v>0.0530344715678392</v>
+      </c>
+      <c r="E16" s="0" t="n">
+        <f aca="false">E10/H10</f>
+        <v>3.51536808020697E-015</v>
+      </c>
+      <c r="F16" s="0" t="n">
+        <f aca="false">F10/I10</f>
+        <v>2436224.4003429</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D17" s="0" t="n">
+        <f aca="false">D11/G11</f>
+        <v>0.23203418452421</v>
+      </c>
+      <c r="E17" s="0" t="n">
+        <f aca="false">E11/H11</f>
+        <v>-4.73358187898108E-017</v>
+      </c>
+      <c r="F17" s="0" t="n">
+        <f aca="false">F11/I11</f>
+        <v>0.0248391335852393</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D18" s="0" t="n">
+        <f aca="false">D12/G12</f>
+        <v>0.516224683696231</v>
+      </c>
+      <c r="E18" s="0" t="n">
+        <f aca="false">E12/H12</f>
+        <v>2.12601129377212E-017</v>
+      </c>
+      <c r="F18" s="0" t="n">
+        <f aca="false">F12/I12</f>
+        <v>1.77187774569047E-016</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D19" s="0" t="n">
+        <f aca="false">D13/G13</f>
+        <v>1888.90729783037</v>
+      </c>
+      <c r="E19" s="0" t="n">
+        <f aca="false">E13/H13</f>
+        <v>-7.2161030697052E-013</v>
+      </c>
+      <c r="F19" s="0" t="n">
+        <f aca="false">F13/I13</f>
+        <v>176.362047635259</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D20" s="0" t="e">
+        <f aca="false">D14/G14</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E20" s="0" t="e">
+        <f aca="false">E14/H14</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="F20" s="0" t="e">
+        <f aca="false">F14/I14</f>
+        <v>#VALUE!</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -975,10 +1217,10 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>11</v>
@@ -1004,10 +1246,10 @@
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>11</v>
@@ -1033,10 +1275,10 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>11</v>
@@ -1062,10 +1304,10 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>27</v>
+        <v>52</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>11</v>
@@ -1091,10 +1333,10 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>11</v>
@@ -1120,10 +1362,10 @@
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>11</v>
@@ -1149,10 +1391,10 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>11</v>
@@ -1178,10 +1420,10 @@
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>34</v>
+        <v>59</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>11</v>
@@ -1207,10 +1449,10 @@
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>36</v>
+        <v>61</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>11</v>
@@ -1236,10 +1478,10 @@
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>39</v>
+        <v>64</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>11</v>
@@ -1306,21 +1548,21 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>43</v>
+        <v>66</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>11</v>
@@ -1346,10 +1588,10 @@
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>45</v>
+        <v>68</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>46</v>
+        <v>69</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>11</v>
@@ -1375,10 +1617,10 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>48</v>
+        <v>71</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>11</v>
@@ -1404,10 +1646,10 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>11</v>
@@ -1433,10 +1675,10 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>11</v>
@@ -1462,10 +1704,10 @@
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>54</v>
+        <v>77</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>11</v>
@@ -1618,13 +1860,13 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D2" s="7" t="n">
         <v>0.999999999999993</v>
@@ -1647,13 +1889,13 @@
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>59</v>
+        <v>82</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D3" s="7" t="n">
         <v>0.96690041040634</v>
@@ -1676,13 +1918,13 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D4" s="7" t="n">
         <v>0.857385186240054</v>
@@ -1705,13 +1947,13 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>63</v>
+        <v>86</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D5" s="9" t="n">
         <v>0.964880939860266</v>
@@ -1734,13 +1976,13 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>64</v>
+        <v>87</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>0.470083098725178</v>
@@ -1763,13 +2005,13 @@
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D7" s="7" t="n">
         <v>0.427133119946537</v>
@@ -1792,13 +2034,13 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>68</v>
+        <v>91</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>69</v>
+        <v>92</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D8" s="7" t="n">
         <v>0.430614670917867</v>
@@ -1821,13 +2063,13 @@
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>71</v>
+        <v>94</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D9" s="7" t="n">
         <v>0.40852653368225</v>
@@ -1850,13 +2092,13 @@
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D10" s="7" t="n">
         <v>0.567821935189133</v>
@@ -1879,13 +2121,13 @@
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D11" s="7" t="n">
         <v>0.492580539472295</v>
@@ -1908,13 +2150,13 @@
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D12" s="7" t="n">
         <v>0.57305721000619</v>
@@ -2140,13 +2382,13 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D2" s="5" t="n">
         <v>0.988927542122776</v>
@@ -2169,13 +2411,13 @@
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D3" s="5" t="n">
         <v>0.827605101501955</v>
@@ -2198,13 +2440,13 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>27</v>
+        <v>52</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D4" s="5" t="n">
         <v>0.766336275007438</v>
@@ -2227,13 +2469,13 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>1.84247411256615E-013</v>
@@ -2256,13 +2498,13 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>82</v>
+        <v>105</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D6" s="5" t="n">
         <v>0.287984724069191</v>
@@ -2319,13 +2561,13 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>83</v>
+        <v>20</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>84</v>
+        <v>21</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>85</v>
+        <v>22</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>6</v>
@@ -2339,13 +2581,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>86</v>
+        <v>106</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>87</v>
+        <v>107</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D2" s="11" t="n">
         <v>0.910665456696755</v>
@@ -2368,13 +2610,13 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>88</v>
+        <v>108</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D3" s="11" t="n">
         <v>0.818007784477811</v>
@@ -2397,13 +2639,13 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>89</v>
+        <v>109</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>46</v>
+        <v>69</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D4" s="11" t="n">
         <v>0.791441912562225</v>
@@ -2426,13 +2668,13 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>48</v>
+        <v>71</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D5" s="11" t="n">
         <v>0.805539978743876</v>
@@ -2455,13 +2697,13 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>91</v>
+        <v>111</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D6" s="11" t="n">
         <v>0.903642482296494</v>
@@ -2484,13 +2726,13 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>93</v>
+        <v>113</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D7" s="11" t="n">
         <v>4.85918015690256E-016</v>
@@ -2513,13 +2755,13 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>94</v>
+        <v>114</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>54</v>
+        <v>77</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D8" s="11" t="n">
         <v>1.23231098938861E-016</v>
@@ -2542,13 +2784,13 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>95</v>
+        <v>115</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>96</v>
+        <v>116</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D9" s="11" t="n">
         <v>3.31969088701663E-013</v>
@@ -2571,13 +2813,13 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>97</v>
+        <v>117</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>98</v>
+        <v>118</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D10" s="11" t="n">
         <v>1.82305832615091E-013</v>
@@ -2600,13 +2842,13 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>99</v>
+        <v>119</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D11" s="11" t="n">
         <v>1.11022302462516E-016</v>
@@ -2629,13 +2871,13 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>101</v>
+        <v>121</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>102</v>
+        <v>122</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D12" s="11" t="n">
         <v>5.55111512312578E-017</v>
@@ -2658,13 +2900,13 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>103</v>
+        <v>123</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>104</v>
+        <v>124</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D13" s="11" t="n">
         <v>0.249547393276211</v>
@@ -2687,13 +2929,13 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>105</v>
+        <v>125</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>106</v>
+        <v>126</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D14" s="11" t="n">
         <v>0.146966848441927</v>
@@ -2716,13 +2958,13 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>107</v>
+        <v>127</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D15" s="11" t="n">
         <v>0.225491878833552</v>
@@ -2745,13 +2987,13 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>109</v>
+        <v>129</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D16" s="11" t="n">
         <v>0.245431174578435</v>
@@ -2774,13 +3016,13 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>111</v>
+        <v>131</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>112</v>
+        <v>132</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D17" s="11" t="n">
         <v>0.277356056970491</v>
@@ -2803,13 +3045,13 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>113</v>
+        <v>133</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>114</v>
+        <v>134</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D18" s="11" t="n">
         <v>0.087648216329556</v>
@@ -2832,13 +3074,13 @@
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>115</v>
+        <v>135</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>116</v>
+        <v>136</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D19" s="11" t="n">
         <v>4.83934632242195E-016</v>
@@ -2861,13 +3103,13 @@
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>117</v>
+        <v>137</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>118</v>
+        <v>138</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D20" s="11" t="n">
         <v>4.55191440096314E-015</v>
@@ -2890,13 +3132,13 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>119</v>
+        <v>139</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D21" s="11" t="n">
         <v>2.60902410786912E-015</v>

</xml_diff>